<commit_message>
Complete Day 21 Sprint 3 validation and retrospective
</commit_message>
<xml_diff>
--- a/output/peer_comparison.xlsx
+++ b/output/peer_comparison.xlsx
@@ -482,7 +482,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -625,7 +625,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>Bajaj Auto Ltd</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -697,7 +697,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>Eicher Motors Ltd</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -769,7 +769,8 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t xml:space="preserve">Hero MotoCorp Ltd
+</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -841,7 +842,8 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t xml:space="preserve">Mahindra &amp; Mahindra Ltd
+</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -913,7 +915,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>Maruti Suzuki India Ltd</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
@@ -985,7 +987,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TATAMOTORS</t>
+          <t>Tata Motors Ltd</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -1045,7 +1047,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TVSMOTOR</t>
+          <t>TVS Motor Company Ltd</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -1193,7 +1195,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -1336,7 +1338,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>Bank of Baroda</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -1408,7 +1410,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CANBK</t>
+          <t>Canara Bank</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -1480,7 +1482,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>Punjab National Bank</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -1534,7 +1536,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>State Bank of India</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr"/>
@@ -1670,7 +1672,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -1813,7 +1815,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>Hindalco Industries Ltd</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -1885,7 +1887,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>JINDALSTEL</t>
+          <t>Jindal Steel &amp; Power Ltd</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -1945,7 +1947,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>JSW Steel Ltd</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -2017,7 +2019,8 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t xml:space="preserve">Tata Steel Ltd
+</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
@@ -2157,7 +2160,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -2300,7 +2303,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>Bajaj Finance Ltd</t>
         </is>
       </c>
       <c r="C2" s="7" t="n">
@@ -2372,7 +2375,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CHOLAFIN</t>
+          <t>Cholamandalam Investment &amp; Finance Company Ltd</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -2444,7 +2447,8 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t xml:space="preserve">Shriram Finance Ltd
+</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -2592,7 +2596,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -2735,7 +2739,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>Britannia Industries Ltd</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -2807,7 +2811,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DABUR</t>
+          <t>Dabur India Ltd</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -2879,7 +2883,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>Godrej Consumer Products Ltd</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -2939,7 +2943,8 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t xml:space="preserve">Hindustan Unilever Ltd
+</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
@@ -3011,7 +3016,8 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t xml:space="preserve">ITC Ltd
+</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -3083,7 +3089,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>Nestle India Ltd</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -3155,7 +3161,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>Tata Consumer Products Ltd</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -3303,7 +3309,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -3446,7 +3452,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>HCL Technologies Ltd</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -3518,7 +3524,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>Infosys Ltd</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -3590,7 +3596,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LTIM</t>
+          <t>LTIMindtree Ltd</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -3662,7 +3668,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>Tata Consultancy Services Ltd</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
@@ -3734,7 +3740,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>Tech Mahindra Ltd</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -3882,7 +3888,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -4025,7 +4031,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>HDFC Life Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -4097,7 +4103,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ICICIPRULI</t>
+          <t>ICICI Prudential Life Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -4169,7 +4175,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>LICI</t>
+          <t>Life Insurance Corporation of India</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
@@ -4237,7 +4243,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>SBI Life Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -4385,7 +4391,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -4528,7 +4534,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>Bharat Petroleum Corporation Ltd</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -4600,7 +4606,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GAIL</t>
+          <t>GAIL (India) Ltd</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -4672,7 +4678,8 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t xml:space="preserve">Indian Oil Corporation
+</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -4744,7 +4751,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>Oil &amp; Natural Gas Corpn Ltd</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -4816,7 +4823,8 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t xml:space="preserve">Reliance Industries Ltd
+</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
@@ -4964,7 +4972,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -5107,7 +5115,8 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t xml:space="preserve">Cipla Ltd
+</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -5179,7 +5188,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>Divis Laboratories Ltd</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -5251,7 +5260,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>Dr Reddys Laboratories Ltd</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -5323,7 +5332,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>Sun Pharmaceuticals Industries Ltd</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
@@ -5395,7 +5404,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TORNTPHARM</t>
+          <t>Torrent Pharmaceuticals Ltd</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -5543,7 +5552,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -5686,7 +5695,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ADANIGREEN</t>
+          <t>Adani Green Energy Ltd</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -5746,7 +5755,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ADANIPOWER</t>
+          <t>Adani Power Ltd</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -5806,7 +5815,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>JSWENERGY</t>
+          <t>JSW Energy Ltd</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -5878,7 +5887,8 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NHPC</t>
+          <t xml:space="preserve">NHPC Ltd
+</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -5950,7 +5960,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>NTPC Ltd</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
@@ -6022,7 +6032,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>Power Grid Corporation of India Ltd</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -6094,7 +6104,8 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t xml:space="preserve">Tata Power Company Ltd
+</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -6242,7 +6253,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -6385,7 +6396,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>Axis Bank Ltd</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -6457,7 +6468,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HDFC Bank Ltd</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
@@ -6529,7 +6540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>ICICI Bank Ltd</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -6601,7 +6612,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>IndusInd Bank Ltd</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -6673,7 +6684,8 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t xml:space="preserve">Kotak Mahindra Bank Ltd
+</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">

</xml_diff>